<commit_message>
feat: minor UX bug fixes — supplier notes, searchable dropdowns, client/supplier history panels
1. Supplier Notes: Added notes field to Supplier model + SupplierHistory audit table
2. Searchable Dropdowns: Replaced all <select> in PO/Quote/Lead forms with SearchableSelect combobox
3. Client History: Added ClientHistoryPanel with History button on ClientsPage
4. Supplier History: Added SupplierHistoryPanel with History button on SuppliersPage
</commit_message>
<xml_diff>
--- a/Initial Inputs/Costerra ERP Task List.xlsx
+++ b/Initial Inputs/Costerra ERP Task List.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeronimo/Documents/Google AntiGravity/Costerra ERP/Initial Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{20462F49-AC15-914F-BE65-B78B3629D3E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B5EA35-16B6-4440-9590-CD82C3DC39A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{9E694293-F02C-FA45-AFB1-414E7BC14C56}"/>
+    <workbookView xWindow="2580" yWindow="500" windowWidth="35820" windowHeight="19520" xr2:uid="{9E694293-F02C-FA45-AFB1-414E7BC14C56}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Task List" sheetId="1" r:id="rId1"/>
+    <sheet name="Tables" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,9 +36,249 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="58">
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Dropped</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Notas Proveedores</t>
+  </si>
+  <si>
+    <t>Agregar campo de "notas" en la sección de proveedores</t>
+  </si>
+  <si>
+    <t>Cambiar Menus Desplegables</t>
+  </si>
+  <si>
+    <t>Cambiar los menús desplegables de selección de proveedores, clientes y cotizaciones por una barra de búsqueda.</t>
+  </si>
+  <si>
+    <t>Implementar la generación de un archivo PDF para las órdenes de compra.</t>
+  </si>
+  <si>
+    <t>Imprimir PDF P.O.</t>
+  </si>
+  <si>
+    <t>Investigar e implementar la funcionalidad de carga de órdenes de compra mediante un archivo Excel/CSV.</t>
+  </si>
+  <si>
+    <t>P.O. con Excel/CSV</t>
+  </si>
+  <si>
+    <t>Diseñar e implementar una función para agregar y prorratear costos adicionales al marcar una orden como "delivered".</t>
+  </si>
+  <si>
+    <t>Manejo de Costos de Importacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Investigar y corregir  la funcionalidad de carga de imágenes de productos.</t>
+  </si>
+  <si>
+    <t>Arreglar Carga de Imagen de Producto</t>
+  </si>
+  <si>
+    <t>Implementar la funcionalidad "make-to-order" para permitir ventas sin stock.</t>
+  </si>
+  <si>
+    <t>Permitir cotizaciones y ventas MTO</t>
+  </si>
+  <si>
+    <t>Añadir la capacidad de gestionar múltiples direcciones para un mismo cliente.</t>
+  </si>
+  <si>
+    <t>Agregar un campo para "Costo de Envío" en las cotizaciones.</t>
+  </si>
+  <si>
+    <t>Permitir la edición de la fecha de validez ("Valid Until") en las cotizaciones.</t>
+  </si>
+  <si>
+    <t>Añadir un botón o estado "Not Sold" para marcar manualmente los leads o cotizaciones perdidas.</t>
+  </si>
+  <si>
+    <t>Agregar la visualización del historial de cambios en los registros de clientes.</t>
+  </si>
+  <si>
+    <t>Implementar la funcionalidad para crear y gestionar "sets" de productos, asegurando el descuento de inventario de sus componentes.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Modificar la exportación del </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>Sales Ledger</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para permitir el análisis de ventas por set y por producto individual.</t>
+    </r>
+  </si>
+  <si>
+    <t>Desarrollar e implementar una función de copias de seguridad automáticas (diarias o al cerrar la app).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Empaquetar la aplicación como un instalador </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>.dmg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> e implementar una función de actualización automática (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>auto-updater</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>Corregir el error visual del botón de la interfaz.</t>
+  </si>
+  <si>
+    <t>Mejorar el flujo de UX: conectar Clientes ; Leads; Cotizaciones para una navegación fluida.</t>
+  </si>
+  <si>
+    <t>Agregar un botón para "cerrar lead". Al cerrar un lead, todas las cotizaciones relacionadas abiertas tienen que pasar a "NOT_SOLD"</t>
+  </si>
+  <si>
+    <t>Corregir registro de ventas para que al vender una cotización todas las demas cotizaciones del mismo lead no pasen a "NOT_SOLD" y no se cierre el lead</t>
+  </si>
+  <si>
+    <t>Corregir flujo de usuario y UX</t>
+  </si>
+  <si>
+    <t>Gestion de dirección de clientes</t>
+  </si>
+  <si>
+    <t>Corregir manejo de costo de envio en cotizaciones</t>
+  </si>
+  <si>
+    <t>Corregir manejo de validez en cotizaciones</t>
+  </si>
+  <si>
+    <t>Corregir exportación de cotizaciones</t>
+  </si>
+  <si>
+    <t>Mejorar la exportación de cotizaciones a Excel para incluir un desglose por producto o set.</t>
+  </si>
+  <si>
+    <t>Corregir estado cotizaciones perdidas</t>
+  </si>
+  <si>
+    <t>Corregir estado automatico de cotizaciones al vender</t>
+  </si>
+  <si>
+    <t>Cerrar leads manualmente y pasar cotizaciones a estado not sold</t>
+  </si>
+  <si>
+    <t>Historial de cambio clientes</t>
+  </si>
+  <si>
+    <t>Gestion de Sets de Productos</t>
+  </si>
+  <si>
+    <t>Task Name</t>
+  </si>
+  <si>
+    <t>Task Description</t>
+  </si>
+  <si>
+    <t>Corregir exportación de sales ledger</t>
+  </si>
+  <si>
+    <t>Backup Automático</t>
+  </si>
+  <si>
+    <t>Installer y Auto Updater</t>
+  </si>
+  <si>
+    <t>Puto boton</t>
+  </si>
+  <si>
+    <t>Historial de cambio proveedores</t>
+  </si>
+  <si>
+    <t>Importancia</t>
+  </si>
+  <si>
+    <t>Crítico</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Medio</t>
+  </si>
+  <si>
+    <t>Bajo</t>
+  </si>
+  <si>
+    <t>Por amor al deporte</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -45,16 +286,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,18 +322,247 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="19">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <u val="double"/>
+        <color rgb="FF5D0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <u val="double"/>
+        <color rgb="FF5D0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <u val="double"/>
+        <color rgb="FF5D0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <u val="double"/>
+        <color rgb="FF5D0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <u val="double"/>
+        <color rgb="FF5D0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF5D0000"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -402,9 +891,631 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1413E950-FABC-C642-9AC2-C8749CBE5FB9}">
-  <dimension ref="A1"/>
+  <dimension ref="B2:G24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="54.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="125.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="1">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="1">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="1">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="1">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="1">
+        <v>7</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="1">
+        <v>8</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="1">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="1">
+        <v>10</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="1">
+        <v>11</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="1">
+        <v>12</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="1">
+        <v>13</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B16" s="1">
+        <v>14</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B17" s="1">
+        <v>15</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B18" s="1">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19" s="1">
+        <v>17</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20" s="1">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="1">
+        <v>19</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B22" s="1">
+        <v>20</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B23" s="1">
+        <v>21</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="1">
+        <v>22</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G24" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="6" operator="equal" id="{DDA78C3B-5CAF-FE48-A683-A23CECA33007}">
+            <xm:f>Tables!$B$6</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="7" operator="equal" id="{ED207B20-18F6-9148-BB9C-142DB625E8C8}">
+            <xm:f>Tables!$B$5</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="8" operator="equal" id="{F8B22381-8055-6A48-AA96-3D6CE6A366DF}">
+            <xm:f>Tables!$B$4</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C5700"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="9" operator="equal" id="{C8B56A3E-411C-B94F-80E9-F698D0D4F7EA}">
+            <xm:f>Tables!$B$3</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>F3:F24</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{BF68C966-3954-F246-905B-7FFA704C067B}">
+            <xm:f>Tables!$D$3</xm:f>
+            <x14:dxf>
+              <font>
+                <b/>
+                <i val="0"/>
+                <u val="double"/>
+                <color rgb="FF5D0000"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{86912034-560C-6E4C-A731-F566207ADB99}">
+            <xm:f>Tables!$D$4</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{27FE812F-6E10-5147-B4E7-3A5B6DB31095}">
+            <xm:f>Tables!$D$5</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C5700"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{D499CFC2-9155-BC4E-86B9-66A2E283B997}">
+            <xm:f>Tables!$D$6</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{B26ECB1D-F812-334D-834B-D307AF490F25}">
+            <xm:f>Tables!$D$7</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E3:E24</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B7056605-1118-B143-8A3F-F6894F4E8E57}">
+          <x14:formula1>
+            <xm:f>Tables!$B$3:$B$6</xm:f>
+          </x14:formula1>
+          <xm:sqref>F3:F24</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7EDE7BB6-818B-F741-B1B0-3C698D3D4B6F}">
+          <x14:formula1>
+            <xm:f>Tables!$D$3:$D$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>E3:E24</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0675A6F2-368D-5F4D-B1BA-B911E24D6758}">
+  <dimension ref="B2:D7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="D7" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: rewrite packaging for production — app now works without Node.js
Root causes fixed:
1. Removed all execSync/npx prisma calls from prisma-client.ts
2. Created schema-bootstrap.ts (raw SQL via better-sqlite3)
3. Added asarUnpack for native modules (.prisma, better-sqlite3, sharp)
4. Added binaryTargets (darwin-arm64, darwin, windows) to Prisma schema
5. Regenerated Prisma client with cross-platform query engines
</commit_message>
<xml_diff>
--- a/Initial Inputs/Costerra ERP Task List.xlsx
+++ b/Initial Inputs/Costerra ERP Task List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeronimo/Documents/Google AntiGravity/Costerra ERP/Initial Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B5EA35-16B6-4440-9590-CD82C3DC39A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3521875-7AFB-3741-A831-507A055EB771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="500" windowWidth="35820" windowHeight="19520" xr2:uid="{9E694293-F02C-FA45-AFB1-414E7BC14C56}"/>
+    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="19520" xr2:uid="{9E694293-F02C-FA45-AFB1-414E7BC14C56}"/>
   </bookViews>
   <sheets>
     <sheet name="Task List" sheetId="1" r:id="rId1"/>
@@ -356,14 +356,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="9">
     <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -379,31 +376,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <u val="double"/>
-        <color rgb="FF5D0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -451,108 +438,9 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <u val="double"/>
-        <color rgb="FF5D0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <u val="double"/>
-        <color rgb="FF5D0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <u val="double"/>
-        <color rgb="FF5D0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -933,7 +821,7 @@
         <v>55</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G3" s="1"/>
     </row>
@@ -951,7 +839,7 @@
         <v>55</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G4" s="1"/>
     </row>
@@ -1203,7 +1091,7 @@
         <v>55</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G18" s="1"/>
     </row>
@@ -1311,7 +1199,7 @@
         <v>55</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G24" s="1"/>
     </row>
@@ -1320,6 +1208,74 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{B26ECB1D-F812-334D-834B-D307AF490F25}">
+            <xm:f>Tables!$D$7</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill>
+                  <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{D499CFC2-9155-BC4E-86B9-66A2E283B997}">
+            <xm:f>Tables!$D$6</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{27FE812F-6E10-5147-B4E7-3A5B6DB31095}">
+            <xm:f>Tables!$D$5</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C5700"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{86912034-560C-6E4C-A731-F566207ADB99}">
+            <xm:f>Tables!$D$4</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{BF68C966-3954-F246-905B-7FFA704C067B}">
+            <xm:f>Tables!$D$3</xm:f>
+            <x14:dxf>
+              <font>
+                <b/>
+                <i val="0"/>
+                <u val="double"/>
+                <color rgb="FF5D0000"/>
+              </font>
+              <fill>
+                <patternFill>
+                  <bgColor rgb="FFFF0000"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>E3:E24</xm:sqref>
+        </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="cellIs" priority="6" operator="equal" id="{DDA78C3B-5CAF-FE48-A683-A23CECA33007}">
             <xm:f>Tables!$B$6</xm:f>
@@ -1372,74 +1328,6 @@
           </x14:cfRule>
           <xm:sqref>F3:F24</xm:sqref>
         </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="equal" id="{BF68C966-3954-F246-905B-7FFA704C067B}">
-            <xm:f>Tables!$D$3</xm:f>
-            <x14:dxf>
-              <font>
-                <b/>
-                <i val="0"/>
-                <u val="double"/>
-                <color rgb="FF5D0000"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFF0000"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="4" operator="equal" id="{86912034-560C-6E4C-A731-F566207ADB99}">
-            <xm:f>Tables!$D$4</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C0006"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFC7CE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="3" operator="equal" id="{27FE812F-6E10-5147-B4E7-3A5B6DB31095}">
-            <xm:f>Tables!$D$5</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C5700"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFFFEB9C"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="2" operator="equal" id="{D499CFC2-9155-BC4E-86B9-66A2E283B997}">
-            <xm:f>Tables!$D$6</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF006100"/>
-              </font>
-              <fill>
-                <patternFill>
-                  <bgColor rgb="FFC6EFCE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{B26ECB1D-F812-334D-834B-D307AF490F25}">
-            <xm:f>Tables!$D$7</xm:f>
-            <x14:dxf>
-              <fill>
-                <patternFill>
-                  <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>E3:E24</xm:sqref>
-        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">

</xml_diff>